<commit_message>
Fix Ufa cost in final top
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/FINAL_TOP_1610.xlsx
+++ b/FINAL_TOP_1610.xlsx
@@ -1448,7 +1448,7 @@
         <v>639849</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>465000</v>
+        <v>373459</v>
       </c>
       <c r="J16" s="17" t="n">
         <v>0.42</v>
@@ -1930,7 +1930,7 @@
         <v>37281482</v>
       </c>
       <c r="I24" s="19" t="n">
-        <v>17536789</v>
+        <v>17445248</v>
       </c>
       <c r="J24" s="18" t="n"/>
       <c r="K24" s="19" t="n">

</xml_diff>

<commit_message>
Rebuild costs on verified 2026 price sources (238 records): COST_REFERENCE_2026, TENDERS_VS_COST, ITOG, tenderer 1-9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/FINAL_TOP_1610.xlsx
+++ b/FINAL_TOP_1610.xlsx
@@ -717,16 +717,16 @@
         <v>6724000</v>
       </c>
       <c r="I4" s="8" t="n">
-        <v>1948000</v>
+        <v>2160000</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.710291493158834</v>
+        <v>0.6787626412849495</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>3108988</v>
+        <v>2922864</v>
       </c>
       <c r="L4" s="9" t="n">
-        <v>0.6983536591937705</v>
+        <v>0.6655256179971993</v>
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
@@ -745,67 +745,67 @@
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>0851300006226000106</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Спецодежда</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>32616431081</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>МКУ «Дзержинка», Новосибирск</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>44-ФЗ аукцион</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>16.10 05:00</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>4400000</v>
-      </c>
-      <c r="I5" s="8" t="n">
-        <v>1724000</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>0.6081818181818182</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>1639990</v>
-      </c>
-      <c r="L5" s="9" t="n">
-        <v>0.5920364158598802</v>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>1% / 5%</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>~400 т × 11 000 ₽/т, МКР | себест. — средняя рыночная с доставкой (не 4 500)</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>высокая</t>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>ФБУ (Госрезерв), 18 позиций</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>223-ФЗ, не аукцион</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>19.10 08:00</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>3637476</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>1366955</v>
+      </c>
+      <c r="J5" s="15" t="n">
+        <v>0.6242022339906012</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>1560296</v>
+      </c>
+      <c r="L5" s="15" t="n">
+        <v>0.6087169747416499</v>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>Цены фабрик Иваново/Тракт; цен за ед. в ЕИС нет — проверить ТЗ</t>
+        </is>
+      </c>
+      <c r="O5" s="11" t="inlineStr">
+        <is>
+          <t>средняя</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>32616431081</t>
+          <t>32616453117</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
@@ -830,33 +830,33 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>ФБУ (Госрезерв), 18 позиций</t>
+          <t>ГУП «Салаватводоканал»</t>
         </is>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>223-ФЗ, не аукцион</t>
+          <t>223-ФЗ запрос предложений</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>19.10 08:00</t>
+          <t>21.10 09:00</t>
         </is>
       </c>
       <c r="H6" s="14" t="n">
-        <v>3637476</v>
+        <v>1500000</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>1460092</v>
+        <v>681523</v>
       </c>
       <c r="J6" s="15" t="n">
-        <v>0.5985975516644549</v>
+        <v>0.5456515118173512</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>1478527</v>
+        <v>539980</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>0.5820572165750648</v>
+        <v>0.5269294629781853</v>
       </c>
       <c r="M6" s="11" t="inlineStr">
         <is>
@@ -865,7 +865,7 @@
       </c>
       <c r="N6" s="11" t="inlineStr">
         <is>
-          <t>Цены фабрик Иваново/Тракт; цен за ед. в ЕИС нет — проверить ТЗ</t>
+          <t>Договор по ед. расценкам</t>
         </is>
       </c>
       <c r="O6" s="11" t="inlineStr">
@@ -912,16 +912,16 @@
         <v>1593800</v>
       </c>
       <c r="I7" s="8" t="n">
-        <v>648700</v>
+        <v>728000</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0.5929853181076672</v>
+        <v>0.5432300163132137</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>572785</v>
+        <v>503164</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>0.5762137232837785</v>
+        <v>0.5244081864507334</v>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
@@ -945,12 +945,12 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Спецодежда</t>
+          <t>ПГР</t>
         </is>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>32616453117</t>
+          <t>32616449090</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -960,502 +960,500 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>ГУП «Салаватводоканал»</t>
+          <t>ГАУК «Мосгортур», Москва</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>223-ФЗ запрос предложений</t>
+          <t>223-ФЗ запрос котировок</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>21.10 09:00</t>
+          <t>19.10 10:00</t>
         </is>
       </c>
       <c r="H8" s="14" t="n">
-        <v>1500000</v>
+        <v>1285964</v>
       </c>
       <c r="I8" s="14" t="n">
-        <v>785120</v>
+        <v>553080</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>0.4765869115363072</v>
+        <v>0.57</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>449028</v>
+        <v>436102</v>
       </c>
       <c r="L8" s="15" t="n">
-        <v>0.4550189616913052</v>
+        <v>0.55</v>
       </c>
       <c r="M8" s="11" t="inlineStr">
         <is>
+          <t>— / 3%</t>
+        </is>
+      </c>
+      <c r="N8" s="11" t="inlineStr">
+        <is>
+          <t>Нужен российский реагент с записью ГИСП</t>
+        </is>
+      </c>
+      <c r="O8" s="11" t="inlineStr">
+        <is>
+          <t>средняя</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Соль</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>0851300006226000106</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>МКУ «Дзержинка», Новосибирск</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>44-ФЗ аукцион</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>16.10 05:00</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>4400000</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>3280000</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>0.2545454545454545</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>273908</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>0.2238279837705378</v>
+      </c>
+      <c r="M9" s="5" t="inlineStr">
+        <is>
+          <t>1% / 5%</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>~400 т × 11 000 ₽/т, МКР | себест. — средняя рыночная с доставкой (не 4 500)</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>высокая</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Арматура</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>32616442935</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>ПАО «Т Плюс», Н.Новгород</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>16.10 14:00</t>
+        </is>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>1883587</v>
+      </c>
+      <c r="I10" s="20" t="n">
+        <v>1273942</v>
+      </c>
+      <c r="J10" s="21" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="K10" s="20" t="n">
+        <v>247436</v>
+      </c>
+      <c r="L10" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
           <t>не указано</t>
         </is>
       </c>
-      <c r="N8" s="11" t="inlineStr">
-        <is>
-          <t>Договор по ед. расценкам</t>
-        </is>
-      </c>
-      <c r="O8" s="11" t="inlineStr">
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Цен по позициям нет — оценка</t>
+        </is>
+      </c>
+      <c r="O10" s="17" t="inlineStr">
+        <is>
+          <t>низкая</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Пробирки</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>0318300254126000157</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>ГБУЗ, Краснодарский край</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>19.10 08:00</t>
+        </is>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>586260</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>184320</v>
+      </c>
+      <c r="J11" s="15" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>208928</v>
+      </c>
+      <c r="L11" s="15" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="M11" s="11" t="inlineStr">
+        <is>
+          <t>— / 5%</t>
+        </is>
+      </c>
+      <c r="N11" s="11" t="inlineStr">
+        <is>
+          <t>Только РФ + РУ; UNIVAC/МиниМед ~9 ₽</t>
+        </is>
+      </c>
+      <c r="O11" s="11" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>ПГР</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>32616449090</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+    <row r="12" ht="32" customHeight="1">
+      <c r="A12" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Спецодежда (коммерч.)</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>4634447</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>ГАУК «Мосгортур», Москва</t>
-        </is>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>223-ФЗ запрос котировок</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>19.10 10:00</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="n">
-        <v>1285964</v>
-      </c>
-      <c r="I9" s="14" t="n">
-        <v>553080</v>
-      </c>
-      <c r="J9" s="15" t="n">
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>ООО «Биннофарм Групп» — пул поставщиков</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
+        <is>
+          <t>Коммерческий запрос предложений</t>
+        </is>
+      </c>
+      <c r="G12" s="17" t="inlineStr">
+        <is>
+          <t>26.10 12:00</t>
+        </is>
+      </c>
+      <c r="H12" s="20" t="n"/>
+      <c r="I12" s="20" t="n">
+        <v>1209448</v>
+      </c>
+      <c r="J12" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K12" s="20" t="n">
+        <v>202731</v>
+      </c>
+      <c r="L12" s="21" t="n">
+        <v>0.2190952275740168</v>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>Без НМЦК: оценка по типовой корзине</t>
+        </is>
+      </c>
+      <c r="O12" s="17" t="inlineStr">
+        <is>
+          <t>низкая</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Соль ⚠ &lt;9 000 ₽/т</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>0128600006826000407</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>МКУ УЖКХ, Струнино</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>19.10</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>1342500</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>870000</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>0.3519553072625698</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>198384</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>0.3252517422613478</v>
+      </c>
+      <c r="M13" s="5" t="inlineStr">
+        <is>
+          <t>1% / 5%</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>Галит тип С, 8 950 ₽/т | себест. — средняя рыночная с доставкой (не 4 500)</t>
+        </is>
+      </c>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>высокая</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Трубы ППУ</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>32616450774</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>МУП «Уфимские инженерные сети»</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>223-ФЗ</t>
+        </is>
+      </c>
+      <c r="G14" s="17" t="inlineStr">
+        <is>
+          <t>20.10 12:00</t>
+        </is>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>639849</v>
+      </c>
+      <c r="I14" s="20" t="n">
+        <v>373459</v>
+      </c>
+      <c r="J14" s="21" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="K14" s="20" t="n">
+        <v>189886</v>
+      </c>
+      <c r="L14" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>не указано</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Отводы ППУ, тяжёлый груз; оценка</t>
+        </is>
+      </c>
+      <c r="O14" s="17" t="inlineStr">
+        <is>
+          <t>низкая</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Пробирки</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>0318300100526000190</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>ГБУЗ «Тихорецкая ЦРБ»</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>44-ФЗ</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>19.10 09:00</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>598970</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>254624</v>
+      </c>
+      <c r="J15" s="15" t="n">
         <v>0.57</v>
       </c>
-      <c r="K9" s="14" t="n">
-        <v>436102</v>
-      </c>
-      <c r="L9" s="15" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="M9" s="11" t="inlineStr">
-        <is>
-          <t>— / 3%</t>
-        </is>
-      </c>
-      <c r="N9" s="11" t="inlineStr">
-        <is>
-          <t>Нужен российский реагент с записью ГИСП</t>
-        </is>
-      </c>
-      <c r="O9" s="11" t="inlineStr">
+      <c r="K15" s="14" t="n">
+        <v>155243</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="M15" s="11" t="inlineStr">
+        <is>
+          <t>— / 5%</t>
+        </is>
+      </c>
+      <c r="N15" s="11" t="inlineStr">
+        <is>
+          <t>Только РФ + РУ</t>
+        </is>
+      </c>
+      <c r="O15" s="11" t="inlineStr">
         <is>
           <t>средняя</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Форма спасателей</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>0358200022926000030</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>ГКУ РО «Ростовская ПСС»</t>
-        </is>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>44-ФЗ аукцион</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>19.10 09:00</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="n">
-        <v>6224421</v>
-      </c>
-      <c r="I10" s="14" t="n">
-        <v>4593594</v>
-      </c>
-      <c r="J10" s="15" t="n">
-        <v>0.2620045749799657</v>
-      </c>
-      <c r="K10" s="14" t="n">
-        <v>323274</v>
-      </c>
-      <c r="L10" s="15" t="n">
-        <v>0.2315944674310844</v>
-      </c>
-      <c r="M10" s="11" t="inlineStr">
-        <is>
-          <t>1% / 10%</t>
-        </is>
-      </c>
-      <c r="N10" s="11" t="inlineStr">
-        <is>
-          <t>Пересчёт по фабричным ценам (комбинезоны 3 766 / ~7 100 ₽); пошив с символикой</t>
-        </is>
-      </c>
-      <c r="O10" s="11" t="inlineStr">
-        <is>
-          <t>средняя</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>0318300065126000256</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>МКУ «Благоустройство», Абинск</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>44-ФЗ аукцион</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>19.10 09:00</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="n">
-        <v>1368000</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>763500</v>
-      </c>
-      <c r="J11" s="9" t="n">
-        <v>0.4418859649122807</v>
-      </c>
-      <c r="K11" s="8" t="n">
-        <v>310162</v>
-      </c>
-      <c r="L11" s="9" t="n">
-        <v>0.4188881152561031</v>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>1% / 5%</t>
-        </is>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>NaCl 96,5–97,7% | себест. — средняя рыночная с доставкой (не 4 500)</t>
-        </is>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>высокая</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Соль ⚠ &lt;9 000 ₽/т</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>0128600006826000407</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>МКУ УЖКХ, Струнино</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>44-ФЗ</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>19.10</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>1342500</v>
-      </c>
-      <c r="I12" s="8" t="n">
-        <v>759000</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <v>0.4346368715083799</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>295836</v>
-      </c>
-      <c r="L12" s="9" t="n">
-        <v>0.4113403130762793</v>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>1% / 5%</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>Галит тип С, 8 950 ₽/т | себест. — средняя рыночная с доставкой (не 4 500)</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>высокая</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="16" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>Арматура</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>32616442935</t>
-        </is>
-      </c>
-      <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E13" s="17" t="inlineStr">
-        <is>
-          <t>ПАО «Т Плюс», Н.Новгород</t>
-        </is>
-      </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="G13" s="17" t="inlineStr">
-        <is>
-          <t>16.10 14:00</t>
-        </is>
-      </c>
-      <c r="H13" s="20" t="n">
-        <v>1883587</v>
-      </c>
-      <c r="I13" s="20" t="n">
-        <v>1273942</v>
-      </c>
-      <c r="J13" s="21" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="K13" s="20" t="n">
-        <v>247436</v>
-      </c>
-      <c r="L13" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="M13" s="17" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="N13" s="17" t="inlineStr">
-        <is>
-          <t>Цен по позициям нет — оценка</t>
-        </is>
-      </c>
-      <c r="O13" s="17" t="inlineStr">
-        <is>
-          <t>низкая</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Пробирки</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>0318300254126000157</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>ГБУЗ, Краснодарский край</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>44-ФЗ</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>19.10 08:00</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="n">
-        <v>586260</v>
-      </c>
-      <c r="I14" s="14" t="n">
-        <v>184320</v>
-      </c>
-      <c r="J14" s="15" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="K14" s="14" t="n">
-        <v>208928</v>
-      </c>
-      <c r="L14" s="15" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="M14" s="11" t="inlineStr">
-        <is>
-          <t>— / 5%</t>
-        </is>
-      </c>
-      <c r="N14" s="11" t="inlineStr">
-        <is>
-          <t>Только РФ + РУ; UNIVAC/МиниМед ~9 ₽</t>
-        </is>
-      </c>
-      <c r="O14" s="11" t="inlineStr">
-        <is>
-          <t>средняя</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="16" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>Трубы ППУ</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>32616450774</t>
-        </is>
-      </c>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="inlineStr">
-        <is>
-          <t>МУП «Уфимские инженерные сети»</t>
-        </is>
-      </c>
-      <c r="F15" s="17" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="G15" s="17" t="inlineStr">
-        <is>
-          <t>20.10 12:00</t>
-        </is>
-      </c>
-      <c r="H15" s="20" t="n">
-        <v>639849</v>
-      </c>
-      <c r="I15" s="20" t="n">
-        <v>373459</v>
-      </c>
-      <c r="J15" s="21" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="K15" s="20" t="n">
-        <v>189886</v>
-      </c>
-      <c r="L15" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="M15" s="17" t="inlineStr">
-        <is>
-          <t>не указано</t>
-        </is>
-      </c>
-      <c r="N15" s="17" t="inlineStr">
-        <is>
-          <t>Отводы ППУ, тяжёлый груз; оценка</t>
-        </is>
-      </c>
-      <c r="O15" s="17" t="inlineStr">
-        <is>
-          <t>низкая</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1468,7 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>0318300100526000190</t>
+          <t>0318300100526000182</t>
         </is>
       </c>
       <c r="D16" s="13" t="inlineStr">
@@ -1490,23 +1488,23 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>19.10 09:00</t>
+          <t>16.10 10:00</t>
         </is>
       </c>
       <c r="H16" s="14" t="n">
-        <v>598970</v>
+        <v>599240</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>254624</v>
+        <v>265328</v>
       </c>
       <c r="J16" s="15" t="n">
-        <v>0.57</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>155243</v>
+        <v>146016</v>
       </c>
       <c r="L16" s="15" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.54</v>
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
@@ -1535,7 +1533,7 @@
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>0318300100526000182</t>
+          <t>0318300100526000186</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -1555,23 +1553,23 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>16.10 10:00</t>
+          <t>20.10 09:00</t>
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>599240</v>
+        <v>597406</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>265328</v>
+        <v>268387</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="K17" s="14" t="n">
-        <v>146016</v>
+        <v>142170</v>
       </c>
       <c r="L17" s="15" t="n">
-        <v>0.54</v>
+        <v>0.53</v>
       </c>
       <c r="M17" s="11" t="inlineStr">
         <is>
@@ -1600,7 +1598,7 @@
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>0318300100526000186</t>
+          <t>0318300100526000191</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -1620,23 +1618,23 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>20.10 09:00</t>
+          <t>21.10 09:00</t>
         </is>
       </c>
       <c r="H18" s="14" t="n">
-        <v>597406</v>
+        <v>598899</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>268387</v>
+        <v>273411</v>
       </c>
       <c r="J18" s="15" t="n">
-        <v>0.55</v>
+        <v>0.54</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>142170</v>
+        <v>138704</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
@@ -1655,311 +1653,325 @@
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Пробирки</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>0318300100526000191</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Спецодежда (коммерч.)</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>372-446</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>ГБУЗ «Тихорецкая ЦРБ»</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>44-ФЗ</t>
-        </is>
-      </c>
-      <c r="G19" s="11" t="inlineStr">
-        <is>
-          <t>21.10 09:00</t>
-        </is>
-      </c>
-      <c r="H19" s="14" t="n">
-        <v>598899</v>
-      </c>
-      <c r="I19" s="14" t="n">
-        <v>273411</v>
-      </c>
-      <c r="J19" s="15" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="K19" s="14" t="n">
-        <v>138704</v>
-      </c>
-      <c r="L19" s="15" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="M19" s="11" t="inlineStr">
-        <is>
-          <t>— / 5%</t>
-        </is>
-      </c>
-      <c r="N19" s="11" t="inlineStr">
-        <is>
-          <t>Только РФ + РУ</t>
-        </is>
-      </c>
-      <c r="O19" s="11" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>ООО «Благо-Армавир»</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>Коммерческий тендер</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>19.10 17:00</t>
+        </is>
+      </c>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n">
+        <v>757377</v>
+      </c>
+      <c r="J19" s="21" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K19" s="20" t="n">
+        <v>126954</v>
+      </c>
+      <c r="L19" s="21" t="n">
+        <v>0.2190952275740167</v>
+      </c>
+      <c r="M19" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N19" s="17" t="inlineStr">
+        <is>
+          <t>Без НМЦК: оценка</t>
+        </is>
+      </c>
+      <c r="O19" s="17" t="inlineStr">
+        <is>
+          <t>низкая</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1">
+      <c r="A20" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>ПГР</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>0372200258526000596</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>СПб ГБУЗ «Больница Св. Георгия»</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>44-ФЗ аукцион</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>20.10</t>
+        </is>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>404960</v>
+      </c>
+      <c r="I20" s="14" t="n">
+        <v>202400</v>
+      </c>
+      <c r="J20" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K20" s="14" t="n">
+        <v>112547</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="M20" s="11" t="inlineStr">
+        <is>
+          <t>— / 10%</t>
+        </is>
+      </c>
+      <c r="N20" s="11" t="inlineStr">
+        <is>
+          <t>ПГРт с мраморной крошкой; ГИСП</t>
+        </is>
+      </c>
+      <c r="O20" s="11" t="inlineStr">
         <is>
           <t>средняя</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="16" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>Спецодежда (коммерч.)</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>4634447</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Соль</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>0318300065126000256</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E20" s="17" t="inlineStr">
-        <is>
-          <t>ООО «Биннофарм Групп» — пул поставщиков</t>
-        </is>
-      </c>
-      <c r="F20" s="17" t="inlineStr">
-        <is>
-          <t>Коммерческий запрос предложений</t>
-        </is>
-      </c>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>26.10 12:00</t>
-        </is>
-      </c>
-      <c r="H20" s="20" t="n"/>
-      <c r="I20" s="20" t="n"/>
-      <c r="J20" s="21" t="n"/>
-      <c r="K20" s="20" t="n">
-        <v>116467</v>
-      </c>
-      <c r="L20" s="21" t="n"/>
-      <c r="M20" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N20" s="17" t="inlineStr">
-        <is>
-          <t>Без НМЦК: оценка по типовой корзине</t>
-        </is>
-      </c>
-      <c r="O20" s="17" t="inlineStr">
-        <is>
-          <t>низкая</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>ПГР</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>0372200258526000596</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>МКУ «Благоустройство», Абинск</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>44-ФЗ аукцион</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>19.10 09:00</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>1368000</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>1050000</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>0.2324561403508772</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>58630</v>
+      </c>
+      <c r="L21" s="9" t="n">
+        <v>0.2008284492716546</v>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>1% / 5%</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>NaCl 96,5–97,7% | себест. — средняя рыночная с доставкой (не 4 500)</t>
+        </is>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>высокая</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Соль ⚠ &lt;9 000 ₽/т</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>0131300000626001316</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>СПб ГБУЗ «Больница Св. Георгия»</t>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>МБУ «Комбинат благоустройства», Воронеж</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>44-ФЗ аукцион</t>
         </is>
       </c>
-      <c r="G21" s="11" t="inlineStr">
-        <is>
-          <t>20.10</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="n">
-        <v>404960</v>
-      </c>
-      <c r="I21" s="14" t="n">
-        <v>202400</v>
-      </c>
-      <c r="J21" s="15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>112547</v>
-      </c>
-      <c r="L21" s="15" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="M21" s="11" t="inlineStr">
-        <is>
-          <t>— / 10%</t>
-        </is>
-      </c>
-      <c r="N21" s="11" t="inlineStr">
-        <is>
-          <t>ПГРт с мраморной крошкой; ГИСП</t>
-        </is>
-      </c>
-      <c r="O21" s="11" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>16.10 09:00</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="n">
+        <v>3296150</v>
+      </c>
+      <c r="I22" s="8" t="n">
+        <v>2996500</v>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>0.09090909090909091</v>
+      </c>
+      <c r="K22" s="8" t="n">
+        <v>-315701</v>
+      </c>
+      <c r="L22" s="9" t="n">
+        <v>0.05344876069577792</v>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>1% / 10%</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>7 150 ₽/т | себест. — средняя рыночная с доставкой (не 4 500)</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>высокая</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Форма спасателей</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>0358200022926000030</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>открыть</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>ГКУ РО «Ростовская ПСС»</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>44-ФЗ аукцион</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>19.10 09:00</t>
+        </is>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>6224421</v>
+      </c>
+      <c r="I23" s="14" t="n">
+        <v>5453674</v>
+      </c>
+      <c r="J23" s="15" t="n">
+        <v>0.1238263088483078</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>-508033</v>
+      </c>
+      <c r="L23" s="15" t="n">
+        <v>0.08772237747407213</v>
+      </c>
+      <c r="M23" s="11" t="inlineStr">
+        <is>
+          <t>1% / 10%</t>
+        </is>
+      </c>
+      <c r="N23" s="11" t="inlineStr">
+        <is>
+          <t>Пересчёт по фабричным ценам (комбинезоны 3 766 / ~7 100 ₽); пошив с символикой</t>
+        </is>
+      </c>
+      <c r="O23" s="11" t="inlineStr">
         <is>
           <t>средняя</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="16" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>Спецодежда (коммерч.)</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>372-446</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E22" s="17" t="inlineStr">
-        <is>
-          <t>ООО «Благо-Армавир»</t>
-        </is>
-      </c>
-      <c r="F22" s="17" t="inlineStr">
-        <is>
-          <t>Коммерческий тендер</t>
-        </is>
-      </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>19.10 17:00</t>
-        </is>
-      </c>
-      <c r="H22" s="20" t="n"/>
-      <c r="I22" s="20" t="n"/>
-      <c r="J22" s="21" t="n"/>
-      <c r="K22" s="20" t="n">
-        <v>99875</v>
-      </c>
-      <c r="L22" s="21" t="n"/>
-      <c r="M22" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="N22" s="17" t="inlineStr">
-        <is>
-          <t>Без НМЦК: оценка</t>
-        </is>
-      </c>
-      <c r="O22" s="17" t="inlineStr">
-        <is>
-          <t>низкая</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1">
-      <c r="A23" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Соль ⚠ &lt;9 000 ₽/т</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>0131300000626001316</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>открыть</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>МБУ «Комбинат благоустройства», Воронеж</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>44-ФЗ аукцион</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>16.10 09:00</t>
-        </is>
-      </c>
-      <c r="H23" s="8" t="n">
-        <v>3296150</v>
-      </c>
-      <c r="I23" s="8" t="n">
-        <v>2839760</v>
-      </c>
-      <c r="J23" s="9" t="n">
-        <v>0.1384615384615385</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>-153808</v>
-      </c>
-      <c r="L23" s="9" t="n">
-        <v>0.102960671674768</v>
-      </c>
-      <c r="M23" s="5" t="inlineStr">
-        <is>
-          <t>1% / 10%</t>
-        </is>
-      </c>
-      <c r="N23" s="5" t="inlineStr">
-        <is>
-          <t>7 150 ₽/т | себест. — средняя рыночная с доставкой (не 4 500)</t>
-        </is>
-      </c>
-      <c r="O23" s="5" t="inlineStr">
-        <is>
-          <t>высокая</t>
         </is>
       </c>
     </row>
@@ -1979,11 +1991,11 @@
         <v>37281482</v>
       </c>
       <c r="I24" s="23" t="n">
-        <v>19170717</v>
+        <v>24202428</v>
       </c>
       <c r="J24" s="24" t="n"/>
       <c r="K24" s="23" t="n">
-        <v>10018156</v>
+        <v>7340209</v>
       </c>
       <c r="L24" s="24" t="n"/>
       <c r="M24" s="24" t="n"/>
@@ -2165,67 +2177,67 @@
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Соль</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>0142200001326018965</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Спецодежда</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>32616425940</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>МБУ «Благоустройство», Самара</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>44-ФЗ аукцион</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>19.10 11:00</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>121000000</v>
-      </c>
-      <c r="I4" s="8" t="n">
-        <v>42350000</v>
-      </c>
-      <c r="J4" s="9" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="K4" s="8" t="n">
-        <v>49542141</v>
-      </c>
-      <c r="L4" s="9" t="n">
-        <v>0.6355777728678744</v>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>0,5% / 0,5%</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>Требуется опыт: исполненный контракт от 24,2 млн; 11 000 т | себест. — средняя рыночная с доставкой (не 4 500)</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>высокая</t>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>ГУП «Петербургский метрополитен»</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>223-ФЗ аукцион</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>16.10 10:00</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>650000000</v>
+      </c>
+      <c r="I4" s="14" t="n">
+        <v>496627641</v>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>39758366</v>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="M4" s="11" t="inlineStr">
+        <is>
+          <t>см. документацию</t>
+        </is>
+      </c>
+      <c r="N4" s="11" t="inlineStr">
+        <is>
+          <t>Рамочный, 1 414 позиций; нужен капитал и гарантии</t>
+        </is>
+      </c>
+      <c r="O4" s="11" t="inlineStr">
+        <is>
+          <t>средняя</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2252,7 @@
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>32616425940</t>
+          <t>32616425363</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -2250,33 +2262,33 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>ГУП «Петербургский метрополитен»</t>
+          <t>АО «Мособлэнерго»</t>
         </is>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>223-ФЗ аукцион</t>
+          <t>223-ФЗ</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>16.10 10:00</t>
+          <t>16.10 11:00</t>
         </is>
       </c>
       <c r="H5" s="14" t="n">
-        <v>650000000</v>
+        <v>200000000</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>496627641</v>
+        <v>133837274</v>
       </c>
       <c r="J5" s="15" t="n">
-        <v>0.22</v>
+        <v>0.32</v>
       </c>
       <c r="K5" s="14" t="n">
-        <v>39758366</v>
+        <v>32511680</v>
       </c>
       <c r="L5" s="15" t="n">
-        <v>0.19</v>
+        <v>0.29</v>
       </c>
       <c r="M5" s="11" t="inlineStr">
         <is>
@@ -2285,7 +2297,7 @@
       </c>
       <c r="N5" s="11" t="inlineStr">
         <is>
-          <t>Рамочный, 1 414 позиций; нужен капитал и гарантии</t>
+          <t>Рамочный; логотип; капитал и гарантии</t>
         </is>
       </c>
       <c r="O5" s="11" t="inlineStr">
@@ -2295,67 +2307,67 @@
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Спецодежда</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>32616425363</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Соль</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>0142200001326018965</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>открыть</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>АО «Мособлэнерго»</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>223-ФЗ</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>16.10 11:00</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="n">
-        <v>200000000</v>
-      </c>
-      <c r="I6" s="14" t="n">
-        <v>133837274</v>
-      </c>
-      <c r="J6" s="15" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="K6" s="14" t="n">
-        <v>32511680</v>
-      </c>
-      <c r="L6" s="15" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="M6" s="11" t="inlineStr">
-        <is>
-          <t>см. документацию</t>
-        </is>
-      </c>
-      <c r="N6" s="11" t="inlineStr">
-        <is>
-          <t>Рамочный; логотип; капитал и гарантии</t>
-        </is>
-      </c>
-      <c r="O6" s="11" t="inlineStr">
-        <is>
-          <t>средняя</t>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>МБУ «Благоустройство», Самара</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>44-ФЗ аукцион</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>19.10 11:00</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>121000000</v>
+      </c>
+      <c r="I6" s="8" t="n">
+        <v>71500000</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0.4090909090909091</v>
+      </c>
+      <c r="K6" s="8" t="n">
+        <v>23950038</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>0.3847416944522556</v>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>0,5% / 0,5%</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>Требуется опыт: исполненный контракт от 24,2 млн; 11 000 т | себест. — средняя рыночная с доставкой (не 4 500)</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>высокая</t>
         </is>
       </c>
     </row>
@@ -2375,11 +2387,11 @@
         <v>971000000</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>672814915</v>
+        <v>701964915</v>
       </c>
       <c r="J7" s="24" t="n"/>
       <c r="K7" s="23" t="n">
-        <v>121812187</v>
+        <v>96220084</v>
       </c>
       <c r="L7" s="24" t="n"/>
       <c r="M7" s="24" t="n"/>

</xml_diff>